<commit_message>
update the other test class with data driven
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataFile.xlsx
+++ b/src/test/resources/TestDataFile.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deven\IdeaProjects\NewFrameworkDesign\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25F42BB6-355E-4C1C-9AEE-D4FB92790E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150F2766-9E7D-4BF8-83E2-2228672E9674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7578867F-E2DE-497D-8A00-BC709CF99601}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{7578867F-E2DE-497D-8A00-BC709CF99601}"/>
   </bookViews>
   <sheets>
     <sheet name="VerifyLogin" sheetId="1" r:id="rId1"/>
     <sheet name="VerifyAdminTab" sheetId="2" r:id="rId2"/>
     <sheet name="VerifyPIMTab" sheetId="3" r:id="rId3"/>
+    <sheet name="VerifyLeaveTab" sheetId="4" r:id="rId4"/>
+    <sheet name="VerifyRecruitmentTab" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="39">
   <si>
     <t>Admin</t>
   </si>
@@ -120,6 +122,39 @@
   </si>
   <si>
     <t>jobTitle</t>
+  </si>
+  <si>
+    <t>leaveType</t>
+  </si>
+  <si>
+    <t>CAN - Personal</t>
+  </si>
+  <si>
+    <t>2025-01-01 - 2025-31-12</t>
+  </si>
+  <si>
+    <t>entitlementValue</t>
+  </si>
+  <si>
+    <t>leavePeriod</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>{faker.email}</t>
+  </si>
+  <si>
+    <t>{faker.contactNum}</t>
+  </si>
+  <si>
+    <t>contactNo</t>
+  </si>
+  <si>
+    <t>vacancy</t>
+  </si>
+  <si>
+    <t>Software Engineer</t>
   </si>
 </sst>
 </file>
@@ -164,7 +199,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -180,6 +215,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -741,4 +779,186 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{617FDAE5-18A0-4DD0-8677-D75D4E89D4D1}">
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" customWidth="1"/>
+    <col min="9" max="9" width="14.5546875" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" customWidth="1"/>
+    <col min="11" max="11" width="22.109375" customWidth="1"/>
+    <col min="12" max="12" width="15.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.109375" customWidth="1"/>
+    <col min="14" max="14" width="18.44140625" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+    </row>
+    <row r="2" spans="1:15" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" s="4">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{0355E16A-D193-4E60-A0D4-E6BAE2C4BA04}"/>
+    <hyperlink ref="I2" r:id="rId2" xr:uid="{87AE9BD4-50CB-4745-B7A1-E0B2601B163E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E4B5182-902B-4FC1-87D1-339D732AD1BD}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>